<commit_message>
chore: add atomic_ops classifier module, scoring notes, and split baseline xlsx files
- New src/mcp_security/atomic_ops/ package: taxonomy, rule engines, classifier,
  discovery, xlsx writer, and server catalog across 16 MCP servers
- Full test suite in tests/atomic_ops/ (8 test files)
- Baseline method xlsx files split into _plain and _security variants for all 7
  methods (chatgpt, cvss_v3, dread, maestro, nist800-30/60, owasp aivss/rr)
- 21 scoring-notes .md files generated (per-method × per-server)
- Updated _fill_xlsx_from_ai.py with multi-mode support; added refill_from_json.py
  and gen_per_server_notes.py helper scripts
- New presentations/atomic_op_classification/ with README and summary xlsx
- Added poster slide template and atomic_operations CSV backup

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/presentations/heatmap_byhand/xlsx/baseline_methods/chatgpt/mcp_sqlite_risk_rankings_chatgpt_plain.xlsx
+++ b/presentations/heatmap_byhand/xlsx/baseline_methods/chatgpt/mcp_sqlite_risk_rankings_chatgpt_plain.xlsx
@@ -71,7 +71,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -112,6 +112,30 @@
       <patternFill patternType="solid">
         <fgColor theme="0"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor rgb="FFFF0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFED7D31"/>
+        <bgColor rgb="FFED7D31"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFD966"/>
+        <bgColor rgb="FFFFD966"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF70AD47"/>
+        <bgColor rgb="FF70AD47"/>
       </patternFill>
     </fill>
   </fills>
@@ -172,7 +196,7 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="2"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -238,6 +262,86 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="4"/>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="3"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -675,32 +779,32 @@
           <t>PII</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E2" s="9" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F2" s="9" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G2" s="9" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="H2" s="21" t="inlineStr">
+      <c r="C2" s="24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D2" s="25" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E2" s="26" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F2" s="26" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G2" s="26" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="H2" s="27" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -717,32 +821,32 @@
           <t>Financial</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E3" s="21" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F3" s="21" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G3" s="21" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="H3" s="10" t="inlineStr">
+      <c r="C3" s="24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D3" s="25" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E3" s="27" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F3" s="27" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G3" s="27" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="H3" s="28" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -759,32 +863,32 @@
           <t>Role / Org</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E4" s="10" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F4" s="10" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G4" s="15" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="H4" s="22" t="inlineStr">
+      <c r="C4" s="24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D4" s="25" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E4" s="28" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F4" s="28" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G4" s="29" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="H4" s="30" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -801,32 +905,32 @@
           <t>Research Metadata</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F5" s="10" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G5" s="15" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H5" s="15" t="inlineStr">
+      <c r="C5" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D5" s="32" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E5" s="32" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F5" s="28" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G5" s="33" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H5" s="33" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -843,32 +947,32 @@
           <t>Timeline</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F6" s="10" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G6" s="15" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H6" s="22" t="inlineStr">
+      <c r="C6" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D6" s="32" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E6" s="32" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F6" s="28" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G6" s="33" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H6" s="34" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -885,32 +989,32 @@
           <t>Public Data</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F7" s="10" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G7" s="15" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H7" s="15" t="inlineStr">
+      <c r="C7" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D7" s="32" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E7" s="32" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F7" s="28" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G7" s="33" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H7" s="33" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -927,32 +1031,32 @@
           <t>Internal Data</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E8" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F8" s="21" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G8" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H8" s="20" t="inlineStr">
+      <c r="C8" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D8" s="32" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E8" s="35" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F8" s="27" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G8" s="35" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H8" s="36" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -969,32 +1073,32 @@
           <t>Research Results</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E9" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F9" s="21" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G9" s="15" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H9" s="10" t="inlineStr">
+      <c r="C9" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D9" s="32" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E9" s="35" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F9" s="27" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G9" s="33" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H9" s="35" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -1011,32 +1115,32 @@
           <t>Public Output</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" s="37" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="38" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G10" s="15" t="inlineStr">
+      <c r="E10" s="32" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F10" s="25" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G10" s="39" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="H10" s="32" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -1053,32 +1157,32 @@
           <t>Financial</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G11" s="9" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="H11" s="21" t="inlineStr">
+      <c r="C11" s="24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D11" s="25" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E11" s="26" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F11" s="26" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G11" s="26" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="H11" s="27" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -1095,32 +1199,32 @@
           <t>Credentials</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G12" s="9" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="H12" s="21" t="inlineStr">
+      <c r="C12" s="24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D12" s="25" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E12" s="26" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F12" s="26" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G12" s="26" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="H12" s="27" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -1193,32 +1297,32 @@
           <t>PII</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="D2" s="9" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E2" s="9" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F2" s="8" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G2" s="17" t="inlineStr">
+      <c r="B2" s="24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="C2" s="25" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D2" s="26" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E2" s="26" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F2" s="40" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G2" s="41" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -1230,32 +1334,32 @@
           <t>Financial</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="D3" s="9" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E3" s="9" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G3" s="18" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="C3" s="25" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D3" s="26" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E3" s="26" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F3" s="40" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G3" s="42" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -1267,32 +1371,32 @@
           <t>Credentials / API Keys</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E4" s="9" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G4" s="8" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="C4" s="25" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D4" s="26" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E4" s="26" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F4" s="26" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G4" s="40" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -1304,32 +1408,32 @@
           <t>Restricted Research Data</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F5" s="18" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="C5" s="25" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D5" s="40" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E5" s="40" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F5" s="42" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G5" s="25" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -1341,32 +1445,32 @@
           <t>Public Research Data</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E6" s="10" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F6" s="19" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G6" s="19" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="C6" s="25" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D6" s="25" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E6" s="28" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F6" s="43" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G6" s="43" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -1378,32 +1482,32 @@
           <t>Org / Role Metadata</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E7" s="10" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G7" s="10" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="C7" s="25" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D7" s="25" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E7" s="28" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F7" s="25" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G7" s="28" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -1415,32 +1519,32 @@
           <t>Lifecycle / Timestamps</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="D8" s="10" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G8" s="10" t="inlineStr">
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="C8" s="25" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D8" s="28" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E8" s="40" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F8" s="25" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G8" s="28" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -1503,32 +1607,32 @@
           <t>employees</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="D2" s="12" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E2" s="9" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G2" s="8" t="inlineStr">
+      <c r="B2" s="24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="C2" s="25" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D2" s="44" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E2" s="26" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F2" s="24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G2" s="40" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -1540,32 +1644,32 @@
           <t>projects</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="D3" s="10" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E3" s="10" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G3" s="15" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="C3" s="25" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D3" s="28" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E3" s="28" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F3" s="24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G3" s="29" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -1577,32 +1681,32 @@
           <t>datasets</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="D4" s="11" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G4" s="10" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="C4" s="25" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D4" s="45" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E4" s="40" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F4" s="24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G4" s="28" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -1614,32 +1718,32 @@
           <t>experiments</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G5" s="15" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="C5" s="25" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D5" s="40" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E5" s="40" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F5" s="24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G5" s="29" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -1651,32 +1755,32 @@
           <t>publications</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E6" s="10" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="C6" s="25" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D6" s="25" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E6" s="28" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F6" s="24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G6" s="25" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -1688,32 +1792,32 @@
           <t>grants</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E7" s="9" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G7" s="16" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="C7" s="25" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D7" s="26" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E7" s="26" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F7" s="24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G7" s="46" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -1725,32 +1829,32 @@
           <t>api_keys</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G8" s="8" t="inlineStr">
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="C8" s="25" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D8" s="26" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E8" s="26" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F8" s="24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G8" s="40" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -1767,12 +1871,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="72" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1791,6 +1896,11 @@
           <t>Risk Level</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Reasoning</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="n">
@@ -1801,9 +1911,14 @@
           <t>list_tables</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" s="38" t="inlineStr">
         <is>
           <t>Medium</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Listing tables can reveal database structure.</t>
         </is>
       </c>
     </row>
@@ -1816,9 +1931,14 @@
           <t>describe_table</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="38" t="inlineStr">
         <is>
           <t>Medium</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Describing tables can expose schema details.</t>
         </is>
       </c>
     </row>
@@ -1831,9 +1951,14 @@
           <t>read_query</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="C4" s="47" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Reading queries can access sensitive data.</t>
         </is>
       </c>
     </row>
@@ -1846,9 +1971,14 @@
           <t>write_query</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="C5" s="40" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Writing queries can alter or delete critical data.</t>
         </is>
       </c>
     </row>
@@ -1861,9 +1991,14 @@
           <t>create_table</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="C6" s="48" t="inlineStr">
         <is>
           <t>Medium</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Creating tables can lead to unauthorized data storage.</t>
         </is>
       </c>
     </row>
@@ -1876,9 +2011,14 @@
           <t>append_insight</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="C7" s="35" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Appending insights can introduce incorrect data.</t>
         </is>
       </c>
     </row>
@@ -1894,12 +2034,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="72" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1918,6 +2059,11 @@
           <t>Risk Level</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Reasoning</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="n">
@@ -1928,9 +2074,14 @@
           <t>PII</t>
         </is>
       </c>
-      <c r="C2" s="9" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="C2" s="26" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>PII exposure can lead to identity theft and privacy issues.</t>
         </is>
       </c>
     </row>
@@ -1943,9 +2094,14 @@
           <t>Financial</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="C3" s="26" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Financial data is highly sensitive and valuable.</t>
         </is>
       </c>
     </row>
@@ -1958,9 +2114,14 @@
           <t>Credentials / API Keys</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="C4" s="26" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Credentials can be used to gain unauthorized access.</t>
         </is>
       </c>
     </row>
@@ -1973,9 +2134,14 @@
           <t>Restricted Research Data</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="C5" s="49" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Restricted data may contain proprietary research.</t>
         </is>
       </c>
     </row>
@@ -1988,9 +2154,14 @@
           <t>Public Research Data</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="38" t="inlineStr">
         <is>
           <t>Medium</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Public data is less sensitive but still valuable.</t>
         </is>
       </c>
     </row>
@@ -2003,9 +2174,14 @@
           <t>Org / Role Metadata</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="48" t="inlineStr">
         <is>
           <t>Medium</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Metadata can reveal organizational insights.</t>
         </is>
       </c>
     </row>
@@ -2018,9 +2194,14 @@
           <t>Lifecycle / Timestamps</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
+      <c r="C8" s="50" t="inlineStr">
         <is>
           <t>Low</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Timestamps generally have low sensitivity.</t>
         </is>
       </c>
     </row>
@@ -2035,12 +2216,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="72" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2059,6 +2241,11 @@
           <t>Risk Level</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Reasoning</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="n">
@@ -2069,9 +2256,14 @@
           <t>employees</t>
         </is>
       </c>
-      <c r="C2" s="12" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="C2" s="44" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Employee table contains sensitive personal information.</t>
         </is>
       </c>
     </row>
@@ -2084,9 +2276,14 @@
           <t>projects</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="C3" s="35" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Project data may include proprietary information.</t>
         </is>
       </c>
     </row>
@@ -2099,9 +2296,14 @@
           <t>datasets</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="C4" s="49" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Datasets can contain sensitive research data.</t>
         </is>
       </c>
     </row>
@@ -2114,9 +2316,14 @@
           <t>experiments</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="C5" s="49" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Experiment data may include confidential research results.</t>
         </is>
       </c>
     </row>
@@ -2129,9 +2336,14 @@
           <t>publications</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="38" t="inlineStr">
         <is>
           <t>Medium</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Publications are generally less sensitive but valuable.</t>
         </is>
       </c>
     </row>
@@ -2144,9 +2356,14 @@
           <t>grants</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="51" t="inlineStr">
         <is>
           <t>Medium</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Grant information can reveal funding sources and amounts.</t>
         </is>
       </c>
     </row>
@@ -2159,9 +2376,14 @@
           <t>api_keys</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="C8" s="26" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>API keys can be used to access systems without authorization.</t>
         </is>
       </c>
     </row>

</xml_diff>